<commit_message>
Direct Write Excel for QC-18 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-18.xlsx
+++ b/FM-MN-07_QC-18.xlsx
@@ -330,7 +330,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -431,6 +431,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1743,7 +1746,11 @@
       <c r="E6" s="26" t="inlineStr"/>
       <c r="F6" s="26" t="inlineStr"/>
       <c r="G6" s="26" t="inlineStr"/>
-      <c r="H6" s="26" t="inlineStr"/>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="26" t="inlineStr"/>
       <c r="J6" s="26" t="inlineStr"/>
       <c r="K6" s="26" t="inlineStr"/>
@@ -1784,7 +1791,11 @@
       <c r="E7" s="26" t="inlineStr"/>
       <c r="F7" s="26" t="inlineStr"/>
       <c r="G7" s="26" t="inlineStr"/>
-      <c r="H7" s="26" t="inlineStr"/>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="26" t="inlineStr"/>
       <c r="J7" s="26" t="inlineStr"/>
       <c r="K7" s="26" t="inlineStr"/>
@@ -1825,7 +1836,11 @@
       <c r="E8" s="26" t="inlineStr"/>
       <c r="F8" s="26" t="inlineStr"/>
       <c r="G8" s="26" t="inlineStr"/>
-      <c r="H8" s="26" t="inlineStr"/>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="26" t="inlineStr"/>
       <c r="J8" s="26" t="inlineStr"/>
       <c r="K8" s="26" t="inlineStr"/>
@@ -1866,7 +1881,11 @@
       <c r="E9" s="26" t="inlineStr"/>
       <c r="F9" s="26" t="inlineStr"/>
       <c r="G9" s="26" t="inlineStr"/>
-      <c r="H9" s="26" t="inlineStr"/>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="26" t="inlineStr"/>
       <c r="J9" s="26" t="inlineStr"/>
       <c r="K9" s="26" t="inlineStr"/>
@@ -1907,7 +1926,11 @@
       <c r="E10" s="26" t="inlineStr"/>
       <c r="F10" s="26" t="inlineStr"/>
       <c r="G10" s="26" t="inlineStr"/>
-      <c r="H10" s="26" t="inlineStr"/>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="26" t="inlineStr"/>
       <c r="J10" s="26" t="inlineStr"/>
       <c r="K10" s="26" t="inlineStr"/>
@@ -1942,7 +1965,11 @@
       <c r="E11" s="38" t="inlineStr"/>
       <c r="F11" s="38" t="inlineStr"/>
       <c r="G11" s="38" t="inlineStr"/>
-      <c r="H11" s="38" t="inlineStr"/>
+      <c r="H11" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ไพรัตน์ </t>
+        </is>
+      </c>
       <c r="I11" s="38" t="inlineStr"/>
       <c r="J11" s="38" t="inlineStr"/>
       <c r="K11" s="38" t="inlineStr"/>
@@ -2079,7 +2106,11 @@
       </c>
     </row>
     <row r="16" ht="185.25" customHeight="1">
-      <c r="B16" s="40" t="inlineStr"/>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>[วันที่ 6]: ข้อ 3: PROBE 3 สึก</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="23.25" customHeight="1"/>
     <row r="18" ht="21" customHeight="1">
@@ -2124,8 +2155,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-18 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-18.xlsx
+++ b/FM-MN-07_QC-18.xlsx
@@ -1754,7 +1754,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="26" t="inlineStr"/>
+      <c r="I6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="26" t="inlineStr"/>
       <c r="K6" s="26" t="inlineStr"/>
       <c r="L6" s="26" t="inlineStr"/>
@@ -1799,7 +1803,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="26" t="inlineStr"/>
+      <c r="I7" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="26" t="inlineStr"/>
       <c r="K7" s="26" t="inlineStr"/>
       <c r="L7" s="26" t="inlineStr"/>
@@ -1844,7 +1852,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="26" t="inlineStr"/>
+      <c r="I8" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="26" t="inlineStr"/>
       <c r="K8" s="26" t="inlineStr"/>
       <c r="L8" s="26" t="inlineStr"/>
@@ -1889,7 +1901,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="26" t="inlineStr"/>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="26" t="inlineStr"/>
       <c r="K9" s="26" t="inlineStr"/>
       <c r="L9" s="26" t="inlineStr"/>
@@ -1934,7 +1950,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="26" t="inlineStr"/>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="26" t="inlineStr"/>
       <c r="K10" s="26" t="inlineStr"/>
       <c r="L10" s="26" t="inlineStr"/>
@@ -1973,7 +1993,11 @@
           <t xml:space="preserve">ไพรัตน์ </t>
         </is>
       </c>
-      <c r="I11" s="38" t="inlineStr"/>
+      <c r="I11" s="41" t="inlineStr">
+        <is>
+          <t>พฤหัส</t>
+        </is>
+      </c>
       <c r="J11" s="38" t="inlineStr"/>
       <c r="K11" s="38" t="inlineStr"/>
       <c r="L11" s="38" t="inlineStr"/>
@@ -2115,7 +2139,7 @@
     <row r="16" ht="185.25" customHeight="1">
       <c r="B16" s="40" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: PROBE 3 สึก</t>
+          <t>[วันที่ 6]: ข้อ 3: PROBE 3 สึก,  [วันที่ 7]: ข้อ 3: หัว3สึกรอแก้ไข</t>
         </is>
       </c>
     </row>
@@ -2162,8 +2186,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-18 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-18.xlsx
+++ b/FM-MN-07_QC-18.xlsx
@@ -1759,7 +1759,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="26" t="inlineStr"/>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="26" t="inlineStr"/>
       <c r="L6" s="26" t="inlineStr"/>
       <c r="M6" s="26" t="inlineStr"/>
@@ -1808,7 +1812,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="26" t="inlineStr"/>
+      <c r="J7" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="26" t="inlineStr"/>
       <c r="L7" s="26" t="inlineStr"/>
       <c r="M7" s="26" t="inlineStr"/>
@@ -1857,7 +1865,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="26" t="inlineStr"/>
+      <c r="J8" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="26" t="inlineStr"/>
       <c r="L8" s="26" t="inlineStr"/>
       <c r="M8" s="26" t="inlineStr"/>
@@ -1906,7 +1918,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="26" t="inlineStr"/>
+      <c r="J9" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="26" t="inlineStr"/>
       <c r="L9" s="26" t="inlineStr"/>
       <c r="M9" s="26" t="inlineStr"/>
@@ -1955,7 +1971,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="26" t="inlineStr"/>
+      <c r="J10" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="26" t="inlineStr"/>
       <c r="L10" s="26" t="inlineStr"/>
       <c r="M10" s="26" t="inlineStr"/>
@@ -1998,7 +2018,11 @@
           <t>พฤหัส</t>
         </is>
       </c>
-      <c r="J11" s="38" t="inlineStr"/>
+      <c r="J11" s="41" t="inlineStr">
+        <is>
+          <t>พฤหัส</t>
+        </is>
+      </c>
       <c r="K11" s="38" t="inlineStr"/>
       <c r="L11" s="38" t="inlineStr"/>
       <c r="M11" s="38" t="inlineStr"/>
@@ -2139,7 +2163,7 @@
     <row r="16" ht="185.25" customHeight="1">
       <c r="B16" s="40" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: PROBE 3 สึก,  [วันที่ 7]: ข้อ 3: หัว3สึกรอแก้ไข</t>
+          <t>[วันที่ 6]: ข้อ 3: PROBE 3 สึก,  [วันที่ 7]: ข้อ 3: หัว3สึกรอแก้ไข,  [วันที่ 8]: ข้อ 3: หัว3สึกรอแก้ไข</t>
         </is>
       </c>
     </row>
@@ -2186,8 +2210,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-18 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-18.xlsx
+++ b/FM-MN-07_QC-18.xlsx
@@ -1765,7 +1765,11 @@
         </is>
       </c>
       <c r="K6" s="26" t="inlineStr"/>
-      <c r="L6" s="26" t="inlineStr"/>
+      <c r="L6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="26" t="inlineStr"/>
       <c r="N6" s="26" t="inlineStr"/>
       <c r="O6" s="26" t="inlineStr"/>
@@ -1818,7 +1822,11 @@
         </is>
       </c>
       <c r="K7" s="26" t="inlineStr"/>
-      <c r="L7" s="26" t="inlineStr"/>
+      <c r="L7" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="26" t="inlineStr"/>
       <c r="N7" s="26" t="inlineStr"/>
       <c r="O7" s="26" t="inlineStr"/>
@@ -1871,7 +1879,11 @@
         </is>
       </c>
       <c r="K8" s="26" t="inlineStr"/>
-      <c r="L8" s="26" t="inlineStr"/>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="26" t="inlineStr"/>
       <c r="N8" s="26" t="inlineStr"/>
       <c r="O8" s="26" t="inlineStr"/>
@@ -1924,7 +1936,11 @@
         </is>
       </c>
       <c r="K9" s="26" t="inlineStr"/>
-      <c r="L9" s="26" t="inlineStr"/>
+      <c r="L9" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="26" t="inlineStr"/>
       <c r="N9" s="26" t="inlineStr"/>
       <c r="O9" s="26" t="inlineStr"/>
@@ -1977,7 +1993,11 @@
         </is>
       </c>
       <c r="K10" s="26" t="inlineStr"/>
-      <c r="L10" s="26" t="inlineStr"/>
+      <c r="L10" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="26" t="inlineStr"/>
       <c r="N10" s="26" t="inlineStr"/>
       <c r="O10" s="26" t="inlineStr"/>
@@ -2024,7 +2044,11 @@
         </is>
       </c>
       <c r="K11" s="38" t="inlineStr"/>
-      <c r="L11" s="38" t="inlineStr"/>
+      <c r="L11" s="41" t="inlineStr">
+        <is>
+          <t>พฤหัส</t>
+        </is>
+      </c>
       <c r="M11" s="38" t="inlineStr"/>
       <c r="N11" s="38" t="inlineStr"/>
       <c r="O11" s="38" t="inlineStr"/>
@@ -2163,7 +2187,7 @@
     <row r="16" ht="185.25" customHeight="1">
       <c r="B16" s="40" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: PROBE 3 สึก,  [วันที่ 7]: ข้อ 3: หัว3สึกรอแก้ไข,  [วันที่ 8]: ข้อ 3: หัว3สึกรอแก้ไข</t>
+          <t>[วันที่ 6]: ข้อ 3: PROBE 3 สึก,  [วันที่ 7]: ข้อ 3: หัว3สึกรอแก้ไข,  [วันที่ 8]: ข้อ 3: หัว3สึกรอแก้ไข,  [วันที่ 10]: ข้อ 3: หัว3สึกรอแก้ไข</t>
         </is>
       </c>
     </row>
@@ -2210,8 +2234,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>